<commit_message>
Further progress on data block definitions autogen
</commit_message>
<xml_diff>
--- a/UniversalDataBlock.xlsx
+++ b/UniversalDataBlock.xlsx
@@ -34,10 +34,10 @@
     <t xml:space="preserve">Units</t>
   </si>
   <si>
-    <t xml:space="preserve">Limit Min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limit Max</t>
+    <t xml:space="preserve">Min Limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Limit</t>
   </si>
   <si>
     <t xml:space="preserve">Default</t>

</xml_diff>